<commit_message>
docs(inventory): reconcile meeting questions with current catalog
</commit_message>
<xml_diff>
--- a/archivos-externos/reuniones/dudas_inventario_por_area.xlsx
+++ b/archivos-externos/reuniones/dudas_inventario_por_area.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="1" r:id="Rc57788c9591f408c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cocina" sheetId="2" r:id="R5490e250f59a4a3d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pastelería" sheetId="3" r:id="R52e125a774194d50"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Panadería" sheetId="4" r:id="R9479437d738d421d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Servicio" sheetId="5" r:id="R210f6525d1c64e0d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bodega Principal" sheetId="6" r:id="Rf0c35a0beba74d3f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="1" r:id="R2d3c57b0ba234bac"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cocina" sheetId="2" r:id="R3447675f9ccc462f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pastelería" sheetId="3" r:id="R73c6549d49b64771"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Panadería" sheetId="4" r:id="Re2797d68181d4bc8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Servicio" sheetId="5" r:id="R36f2dad29ca84486"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bodega Principal" sheetId="6" r:id="R782689ceeb3d4886"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -192,7 +192,7 @@
         <x:color rgb="FF92400E"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEF3C7"/>
         </x:patternFill>
       </x:fill>
@@ -202,7 +202,7 @@
         <x:color rgb="FF166534"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFDCFCE7"/>
         </x:patternFill>
       </x:fill>
@@ -212,7 +212,7 @@
         <x:color rgb="FF92400E"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEF3C7"/>
         </x:patternFill>
       </x:fill>
@@ -222,7 +222,7 @@
         <x:color rgb="FF166534"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFDCFCE7"/>
         </x:patternFill>
       </x:fill>
@@ -232,7 +232,7 @@
         <x:color rgb="FF92400E"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEF3C7"/>
         </x:patternFill>
       </x:fill>
@@ -242,7 +242,7 @@
         <x:color rgb="FF166534"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFDCFCE7"/>
         </x:patternFill>
       </x:fill>
@@ -252,7 +252,7 @@
         <x:color rgb="FF92400E"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEF3C7"/>
         </x:patternFill>
       </x:fill>
@@ -262,7 +262,7 @@
         <x:color rgb="FF166534"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFDCFCE7"/>
         </x:patternFill>
       </x:fill>
@@ -272,7 +272,7 @@
         <x:color rgb="FF92400E"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEF3C7"/>
         </x:patternFill>
       </x:fill>
@@ -282,7 +282,7 @@
         <x:color rgb="FF166534"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFDCFCE7"/>
         </x:patternFill>
       </x:fill>
@@ -754,11 +754,11 @@
       </x:c>
       <x:c r="B10" s="28" t="n">
         <x:f>COUNTIF('Servicio'!$C$6:$C$100,"&lt;&gt;")</x:f>
-        <x:v>34</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="C10" s="28" t="n">
         <x:f>COUNTIFS('Servicio'!$C$6:$C$100,"&lt;&gt;",'Servicio'!$A$6:$A$100,"Pendiente")</x:f>
-        <x:v>34</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="D10" s="28" t="n">
         <x:f>COUNTIFS('Servicio'!$C$6:$C$100,"&lt;&gt;",'Servicio'!$A$6:$A$100,"En revisión")</x:f>
@@ -804,11 +804,11 @@
       </x:c>
       <x:c r="B12" s="29" t="n">
         <x:f>SUM(B7:B11)</x:f>
-        <x:v>129</x:v>
+        <x:v>130</x:v>
       </x:c>
       <x:c r="C12" s="29" t="n">
         <x:f>SUM(C7:C11)</x:f>
-        <x:v>129</x:v>
+        <x:v>130</x:v>
       </x:c>
       <x:c r="D12" s="29" t="n">
         <x:f>SUM(D7:D11)</x:f>
@@ -1167,7 +1167,7 @@
         <x:v>Abarrotes</x:v>
       </x:c>
       <x:c r="I7" s="11" t="str">
-        <x:v>Verduras, frutas y hierbas</x:v>
+        <x:v>Verduras y frutas</x:v>
       </x:c>
       <x:c r="J7" s="10" t="str">
         <x:v>¿La categoría de conteo debe ser Abarrotes o Verduras, frutas y hierbas?</x:v>
@@ -1238,7 +1238,7 @@
         <x:v>Hoy muestra y guarda KG; factor configurado 1:1.</x:v>
       </x:c>
       <x:c r="H9" s="10" t="str">
-        <x:v>Verduras, frutas y hierbas</x:v>
+        <x:v>Verduras y frutas</x:v>
       </x:c>
       <x:c r="I9" s="11" t="str"/>
       <x:c r="J9" s="10" t="str">
@@ -1274,7 +1274,7 @@
         <x:v>Hoy muestra y guarda UN; factor configurado 1:1.</x:v>
       </x:c>
       <x:c r="H10" s="10" t="str">
-        <x:v>Verduras, frutas y hierbas</x:v>
+        <x:v>Verduras y frutas</x:v>
       </x:c>
       <x:c r="I10" s="11" t="str"/>
       <x:c r="J10" s="10" t="str">
@@ -2105,7 +2105,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra9313321bfc24e7c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R413121470e8b41f6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2256,7 +2256,7 @@
         <x:v>Galleta alfajor</x:v>
       </x:c>
       <x:c r="D6" s="13" t="str">
-        <x:v>Por definir: UN/GR/KG</x:v>
+        <x:v>Sin definir</x:v>
       </x:c>
       <x:c r="E6" s="16" t="str"/>
       <x:c r="F6" s="13" t="str"/>
@@ -2290,7 +2290,7 @@
         <x:v>Galleta alfajor</x:v>
       </x:c>
       <x:c r="D7" s="13" t="str">
-        <x:v>Por definir: UN/GR/KG</x:v>
+        <x:v>Sin definir</x:v>
       </x:c>
       <x:c r="E7" s="16" t="str"/>
       <x:c r="F7" s="13" t="str"/>
@@ -2326,7 +2326,7 @@
         <x:v>Relleno Lotus</x:v>
       </x:c>
       <x:c r="D8" s="13" t="str">
-        <x:v>Por definir: GR/KG/UN</x:v>
+        <x:v>Sin definir</x:v>
       </x:c>
       <x:c r="E8" s="16" t="str"/>
       <x:c r="F8" s="13" t="str"/>
@@ -2358,7 +2358,7 @@
         <x:v>ganache pistacho</x:v>
       </x:c>
       <x:c r="D9" s="13" t="str">
-        <x:v>Por definir: GR/KG</x:v>
+        <x:v>Sin definir</x:v>
       </x:c>
       <x:c r="E9" s="16" t="str"/>
       <x:c r="F9" s="13" t="str"/>
@@ -2390,7 +2390,7 @@
         <x:v>ganache pistacho</x:v>
       </x:c>
       <x:c r="D10" s="13" t="str">
-        <x:v>Por definir: GR/KG</x:v>
+        <x:v>Sin definir</x:v>
       </x:c>
       <x:c r="E10" s="16" t="str"/>
       <x:c r="F10" s="13" t="str"/>
@@ -2424,7 +2424,7 @@
         <x:v>ganache de chocolate sin azucar </x:v>
       </x:c>
       <x:c r="D11" s="13" t="str">
-        <x:v>Por definir: GR/KG</x:v>
+        <x:v>Sin definir</x:v>
       </x:c>
       <x:c r="E11" s="16" t="str"/>
       <x:c r="F11" s="13" t="str"/>
@@ -2456,7 +2456,7 @@
         <x:v>ganache de chocolate sin azucar </x:v>
       </x:c>
       <x:c r="D12" s="13" t="str">
-        <x:v>Por definir: GR/KG</x:v>
+        <x:v>Sin definir</x:v>
       </x:c>
       <x:c r="E12" s="16" t="str"/>
       <x:c r="F12" s="13" t="str"/>
@@ -2490,7 +2490,7 @@
         <x:v>Salsa frutos rojos sin azucar</x:v>
       </x:c>
       <x:c r="D13" s="13" t="str">
-        <x:v>Por definir: GR/KG/CC</x:v>
+        <x:v>Sin definir</x:v>
       </x:c>
       <x:c r="E13" s="16" t="str"/>
       <x:c r="F13" s="13" t="str"/>
@@ -2563,14 +2563,14 @@
       </x:c>
       <x:c r="F15" s="13" t="str"/>
       <x:c r="G15" s="13" t="str">
-        <x:v>Muestra dos filas separadas y guarda UN en cada una.</x:v>
+        <x:v>La app muestra dos filas separadas en Pastelería; Mercadito repite los mismos dos ID.</x:v>
       </x:c>
       <x:c r="H15" s="10" t="str">
         <x:v>Tortas y moldes</x:v>
       </x:c>
       <x:c r="I15" s="11" t="str"/>
       <x:c r="J15" s="10" t="str">
-        <x:v>¿Son dos productos distintos o el mismo stock con ID diferentes? ¿Cómo se asigna a cada fila?</x:v>
+        <x:v>¿Son dos productos distintos? Si sí, ¿cómo los distingue el equipo? Si es uno solo, ¿a cuál ID/fila se asigna el conteo?</x:v>
       </x:c>
       <x:c r="K15" s="13" t="str"/>
       <x:c r="L15" s="15" t="str">
@@ -2579,7 +2579,9 @@
       <x:c r="M15" s="2" t="str">
         <x:v>ti-ing-eb1667ba-d42f-482b-b42e-0a4c9806ac59 / ti-ing-4dac4d03-1043-4a27-a1e1-ed68340239cb</x:v>
       </x:c>
-      <x:c r="N15" s="14" t="str"/>
+      <x:c r="N15" s="14" t="str">
+        <x:v>También en Servicio/Mercadito, filas 273 y 274.</x:v>
+      </x:c>
     </x:row>
     <x:row r="16" ht="62" customHeight="1">
       <x:c r="A16" s="2" t="str">
@@ -4056,7 +4058,7 @@
         <x:v>Relleno Lotus</x:v>
       </x:c>
       <x:c r="D59" s="13" t="str">
-        <x:v>Por definir: GR/KG/UN</x:v>
+        <x:v>Sin definir</x:v>
       </x:c>
       <x:c r="E59" s="16" t="str"/>
       <x:c r="F59" s="13" t="str"/>
@@ -4088,7 +4090,7 @@
         <x:v>ganache pistacho</x:v>
       </x:c>
       <x:c r="D60" s="13" t="str">
-        <x:v>Por definir: GR/KG</x:v>
+        <x:v>Sin definir</x:v>
       </x:c>
       <x:c r="E60" s="16" t="str"/>
       <x:c r="F60" s="13" t="str"/>
@@ -4120,7 +4122,7 @@
         <x:v>ganache de chocolate sin azucar </x:v>
       </x:c>
       <x:c r="D61" s="13" t="str">
-        <x:v>Por definir: GR/KG</x:v>
+        <x:v>Sin definir</x:v>
       </x:c>
       <x:c r="E61" s="16" t="str"/>
       <x:c r="F61" s="13" t="str"/>
@@ -4186,7 +4188,7 @@
         <x:v>Salsa frutos rojos sin azucar</x:v>
       </x:c>
       <x:c r="D63" s="13" t="str">
-        <x:v>Por definir: GR/KG/CC</x:v>
+        <x:v>Sin definir</x:v>
       </x:c>
       <x:c r="E63" s="16" t="str"/>
       <x:c r="F63" s="13" t="str"/>
@@ -4443,7 +4445,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R18d12c54d27c4a57"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7790e4206d8f48ec"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4816,7 +4818,7 @@
         <x:v>Hoy conserva el ID GetJusto vacío y vincula el conteo por hoja y fila.</x:v>
       </x:c>
       <x:c r="H12" s="10" t="str">
-        <x:v>Harinas, levaduras y mejoradores</x:v>
+        <x:v>Harinas y levaduras</x:v>
       </x:c>
       <x:c r="I12" s="11" t="str"/>
       <x:c r="J12" s="10" t="str">
@@ -5065,7 +5067,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R61db0abcee8c4c79"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R57adef1cb56845db"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5310,70 +5312,74 @@
         <x:v>Pendiente</x:v>
       </x:c>
       <x:c r="B8" s="2" t="str">
-        <x:v>Ubicación de conteo</x:v>
+        <x:v>Producto duplicado</x:v>
       </x:c>
       <x:c r="C8" s="10" t="str">
-        <x:v>Marca VITRINA (41 productos)</x:v>
+        <x:v>Torta Manjar nuez / Torta manjar nuez</x:v>
       </x:c>
       <x:c r="D8" s="10" t="str">
         <x:v>Mercadito</x:v>
       </x:c>
-      <x:c r="E8" s="10" t="str"/>
-      <x:c r="F8" s="13" t="str"/>
-      <x:c r="G8" s="16" t="str"/>
-      <x:c r="H8" s="13" t="str"/>
+      <x:c r="E8" s="10"/>
+      <x:c r="F8" s="13" t="str">
+        <x:v>UN</x:v>
+      </x:c>
+      <x:c r="G8" s="16" t="str">
+        <x:v>UN / UN</x:v>
+      </x:c>
+      <x:c r="H8" s="13"/>
       <x:c r="I8" s="13" t="str">
-        <x:v>Marca de VITRINA registrada en el listado manual; por confirmar su alcance.</x:v>
+        <x:v>La app muestra dos ítems separados y guarda cada conteo en su fila.</x:v>
       </x:c>
       <x:c r="J8" s="10" t="str">
-        <x:v>Productos de vitrina</x:v>
-      </x:c>
-      <x:c r="K8" s="11" t="str"/>
+        <x:v>Productos Elaborados</x:v>
+      </x:c>
+      <x:c r="K8" s="11"/>
       <x:c r="L8" s="10" t="str">
-        <x:v>¿La marca VITRINA indica aún dónde se cuentan esos 41 productos? ¿Hay productos no marcados que también se guardan ahí?</x:v>
-      </x:c>
-      <x:c r="M8" s="13" t="str"/>
-      <x:c r="N8" s="15" t="str"/>
-      <x:c r="O8" s="2" t="str"/>
-      <x:c r="P8" s="14" t="str"/>
+        <x:v>¿Cómo distingue Mercadito estas dos tortas? Si son el mismo producto, ¿a cuál ID/fila se asigna su stock?</x:v>
+      </x:c>
+      <x:c r="M8" s="13"/>
+      <x:c r="N8" s="15" t="str">
+        <x:v>273, 274</x:v>
+      </x:c>
+      <x:c r="O8" s="2" t="str">
+        <x:v>ti-ing-eb1667ba-d42f-482b-b42e-0a4c9806ac59 / ti-ing-4dac4d03-1043-4a27-a1e1-ed68340239cb</x:v>
+      </x:c>
+      <x:c r="P8" s="14" t="str">
+        <x:v>Mismos dos ID en Pastelería, filas 230 y 231.</x:v>
+      </x:c>
     </x:row>
     <x:row r="9" ht="62" customHeight="1">
       <x:c r="A9" s="2" t="str">
         <x:v>Pendiente</x:v>
       </x:c>
       <x:c r="B9" s="2" t="str">
-        <x:v>ID GetJusto</x:v>
+        <x:v>Ubicación de conteo</x:v>
       </x:c>
       <x:c r="C9" s="10" t="str">
-        <x:v>Primaveral</x:v>
+        <x:v>Marca VITRINA (41 productos)</x:v>
       </x:c>
       <x:c r="D9" s="10" t="str">
-        <x:v>Barra</x:v>
-      </x:c>
-      <x:c r="E9" s="10" t="str"/>
-      <x:c r="F9" s="13" t="str">
-        <x:v>UN</x:v>
-      </x:c>
-      <x:c r="G9" s="16" t="str">
-        <x:v>UN</x:v>
-      </x:c>
-      <x:c r="H9" s="13" t="str"/>
+        <x:v>Mercadito</x:v>
+      </x:c>
+      <x:c r="E9" s="10"/>
+      <x:c r="F9" s="13"/>
+      <x:c r="G9" s="16"/>
+      <x:c r="H9" s="13"/>
       <x:c r="I9" s="13" t="str">
-        <x:v>Conserva el ID GetJusto vacío y vincula por hoja y fila.</x:v>
+        <x:v>La app carga 139 ítems en Mercadito; el listado manual marca 41 como VITRINA.</x:v>
       </x:c>
       <x:c r="J9" s="10" t="str">
-        <x:v>Bebestibles</x:v>
-      </x:c>
-      <x:c r="K9" s="11" t="str"/>
+        <x:v>No aplica: criterio de ubicación</x:v>
+      </x:c>
+      <x:c r="K9" s="11"/>
       <x:c r="L9" s="10" t="str">
-        <x:v>¿Tiene un ID GetJusto vigente? Si existe, ¿cuál? Si no, confirmar que esta fila queda sin ID.</x:v>
-      </x:c>
-      <x:c r="M9" s="13" t="str"/>
-      <x:c r="N9" s="15" t="str">
-        <x:v>62</x:v>
-      </x:c>
-      <x:c r="O9" s="2" t="str"/>
-      <x:c r="P9" s="14" t="str"/>
+        <x:v>¿Cuáles de los 139 ítems cargados se guardan en Mercadito? ¿Sigue vigente la marca VITRINA de 41 productos?</x:v>
+      </x:c>
+      <x:c r="M9" s="13"/>
+      <x:c r="N9" s="15"/>
+      <x:c r="O9" s="2"/>
+      <x:c r="P9" s="14"/>
     </x:row>
     <x:row r="10" ht="62" customHeight="1">
       <x:c r="A10" s="2" t="str">
@@ -5383,35 +5389,35 @@
         <x:v>ID GetJusto</x:v>
       </x:c>
       <x:c r="C10" s="10" t="str">
-        <x:v>Frutillas</x:v>
+        <x:v>Primaveral</x:v>
       </x:c>
       <x:c r="D10" s="10" t="str">
         <x:v>Barra</x:v>
       </x:c>
-      <x:c r="E10" s="10" t="str"/>
+      <x:c r="E10" s="10"/>
       <x:c r="F10" s="13" t="str">
-        <x:v>KG</x:v>
+        <x:v>UN</x:v>
       </x:c>
       <x:c r="G10" s="16" t="str">
-        <x:v>KG</x:v>
-      </x:c>
-      <x:c r="H10" s="13" t="str"/>
+        <x:v>UN</x:v>
+      </x:c>
+      <x:c r="H10" s="13"/>
       <x:c r="I10" s="13" t="str">
         <x:v>Conserva el ID GetJusto vacío y vincula por hoja y fila.</x:v>
       </x:c>
       <x:c r="J10" s="10" t="str">
-        <x:v>Frutas y Verduras</x:v>
-      </x:c>
-      <x:c r="K10" s="11" t="str"/>
+        <x:v>Insumos</x:v>
+      </x:c>
+      <x:c r="K10" s="11"/>
       <x:c r="L10" s="10" t="str">
         <x:v>¿Tiene un ID GetJusto vigente? Si existe, ¿cuál? Si no, confirmar que esta fila queda sin ID.</x:v>
       </x:c>
-      <x:c r="M10" s="13" t="str"/>
+      <x:c r="M10" s="13"/>
       <x:c r="N10" s="15" t="str">
-        <x:v>137</x:v>
-      </x:c>
-      <x:c r="O10" s="2" t="str"/>
-      <x:c r="P10" s="14" t="str"/>
+        <x:v>62</x:v>
+      </x:c>
+      <x:c r="O10" s="2"/>
+      <x:c r="P10" s="14"/>
     </x:row>
     <x:row r="11" ht="62" customHeight="1">
       <x:c r="A11" s="2" t="str">
@@ -5421,35 +5427,35 @@
         <x:v>ID GetJusto</x:v>
       </x:c>
       <x:c r="C11" s="10" t="str">
-        <x:v>Infusión té flor de jamaica</x:v>
+        <x:v>Frutillas</x:v>
       </x:c>
       <x:c r="D11" s="10" t="str">
         <x:v>Barra</x:v>
       </x:c>
-      <x:c r="E11" s="10" t="str"/>
+      <x:c r="E11" s="10"/>
       <x:c r="F11" s="13" t="str">
-        <x:v>LT</x:v>
+        <x:v>KG</x:v>
       </x:c>
       <x:c r="G11" s="16" t="str">
-        <x:v>LT</x:v>
-      </x:c>
-      <x:c r="H11" s="13" t="str"/>
+        <x:v>KG</x:v>
+      </x:c>
+      <x:c r="H11" s="13"/>
       <x:c r="I11" s="13" t="str">
         <x:v>Conserva el ID GetJusto vacío y vincula por hoja y fila.</x:v>
       </x:c>
       <x:c r="J11" s="10" t="str">
-        <x:v>Productos Elaborados</x:v>
-      </x:c>
-      <x:c r="K11" s="11" t="str"/>
+        <x:v>Insumos</x:v>
+      </x:c>
+      <x:c r="K11" s="11"/>
       <x:c r="L11" s="10" t="str">
         <x:v>¿Tiene un ID GetJusto vigente? Si existe, ¿cuál? Si no, confirmar que esta fila queda sin ID.</x:v>
       </x:c>
-      <x:c r="M11" s="13" t="str"/>
+      <x:c r="M11" s="13"/>
       <x:c r="N11" s="15" t="str">
-        <x:v>225</x:v>
-      </x:c>
-      <x:c r="O11" s="2" t="str"/>
-      <x:c r="P11" s="14" t="str"/>
+        <x:v>137</x:v>
+      </x:c>
+      <x:c r="O11" s="2"/>
+      <x:c r="P11" s="14"/>
     </x:row>
     <x:row r="12" ht="62" customHeight="1">
       <x:c r="A12" s="2" t="str">
@@ -5459,35 +5465,35 @@
         <x:v>ID GetJusto</x:v>
       </x:c>
       <x:c r="C12" s="10" t="str">
-        <x:v>Infusión té mariposa</x:v>
+        <x:v>Infusión té flor de jamaica</x:v>
       </x:c>
       <x:c r="D12" s="10" t="str">
         <x:v>Barra</x:v>
       </x:c>
-      <x:c r="E12" s="10" t="str"/>
+      <x:c r="E12" s="10"/>
       <x:c r="F12" s="13" t="str">
         <x:v>LT</x:v>
       </x:c>
       <x:c r="G12" s="16" t="str">
         <x:v>LT</x:v>
       </x:c>
-      <x:c r="H12" s="13" t="str"/>
+      <x:c r="H12" s="13"/>
       <x:c r="I12" s="13" t="str">
         <x:v>Conserva el ID GetJusto vacío y vincula por hoja y fila.</x:v>
       </x:c>
       <x:c r="J12" s="10" t="str">
-        <x:v>Productos Elaborados</x:v>
-      </x:c>
-      <x:c r="K12" s="11" t="str"/>
+        <x:v>Te / Infusiones</x:v>
+      </x:c>
+      <x:c r="K12" s="11"/>
       <x:c r="L12" s="10" t="str">
         <x:v>¿Tiene un ID GetJusto vigente? Si existe, ¿cuál? Si no, confirmar que esta fila queda sin ID.</x:v>
       </x:c>
-      <x:c r="M12" s="13" t="str"/>
+      <x:c r="M12" s="13"/>
       <x:c r="N12" s="15" t="str">
-        <x:v>226</x:v>
-      </x:c>
-      <x:c r="O12" s="2" t="str"/>
-      <x:c r="P12" s="14" t="str"/>
+        <x:v>225</x:v>
+      </x:c>
+      <x:c r="O12" s="2"/>
+      <x:c r="P12" s="14"/>
     </x:row>
     <x:row r="13" ht="62" customHeight="1">
       <x:c r="A13" s="2" t="str">
@@ -5497,35 +5503,35 @@
         <x:v>ID GetJusto</x:v>
       </x:c>
       <x:c r="C13" s="10" t="str">
-        <x:v>Limonada</x:v>
+        <x:v>Infusión té mariposa</x:v>
       </x:c>
       <x:c r="D13" s="10" t="str">
-        <x:v>Mercadito</x:v>
-      </x:c>
-      <x:c r="E13" s="10" t="str"/>
+        <x:v>Barra</x:v>
+      </x:c>
+      <x:c r="E13" s="10"/>
       <x:c r="F13" s="13" t="str">
         <x:v>LT</x:v>
       </x:c>
       <x:c r="G13" s="16" t="str">
         <x:v>LT</x:v>
       </x:c>
-      <x:c r="H13" s="13" t="str"/>
+      <x:c r="H13" s="13"/>
       <x:c r="I13" s="13" t="str">
         <x:v>Conserva el ID GetJusto vacío y vincula por hoja y fila.</x:v>
       </x:c>
       <x:c r="J13" s="10" t="str">
-        <x:v>Productos Elaborados</x:v>
-      </x:c>
-      <x:c r="K13" s="11" t="str"/>
+        <x:v>Te / Infusiones</x:v>
+      </x:c>
+      <x:c r="K13" s="11"/>
       <x:c r="L13" s="10" t="str">
         <x:v>¿Tiene un ID GetJusto vigente? Si existe, ¿cuál? Si no, confirmar que esta fila queda sin ID.</x:v>
       </x:c>
-      <x:c r="M13" s="13" t="str"/>
+      <x:c r="M13" s="13"/>
       <x:c r="N13" s="15" t="str">
-        <x:v>232</x:v>
-      </x:c>
-      <x:c r="O13" s="2" t="str"/>
-      <x:c r="P13" s="14" t="str"/>
+        <x:v>226</x:v>
+      </x:c>
+      <x:c r="O13" s="2"/>
+      <x:c r="P13" s="14"/>
     </x:row>
     <x:row r="14" ht="62" customHeight="1">
       <x:c r="A14" s="2" t="str">
@@ -5535,41 +5541,35 @@
         <x:v>ID GetJusto</x:v>
       </x:c>
       <x:c r="C14" s="10" t="str">
-        <x:v>Helado frutilla</x:v>
+        <x:v>Limonada</x:v>
       </x:c>
       <x:c r="D14" s="10" t="str">
-        <x:v>Barra</x:v>
-      </x:c>
-      <x:c r="E14" s="10" t="str"/>
+        <x:v>Mercadito</x:v>
+      </x:c>
+      <x:c r="E14" s="10"/>
       <x:c r="F14" s="13" t="str">
-        <x:v>Lt</x:v>
+        <x:v>LT</x:v>
       </x:c>
       <x:c r="G14" s="16" t="str">
         <x:v>LT</x:v>
       </x:c>
-      <x:c r="H14" s="13" t="str">
-        <x:v>1:1</x:v>
-      </x:c>
+      <x:c r="H14" s="13"/>
       <x:c r="I14" s="13" t="str">
         <x:v>Conserva el ID GetJusto vacío y vincula por hoja y fila.</x:v>
       </x:c>
       <x:c r="J14" s="10" t="str">
-        <x:v>Congelados</x:v>
-      </x:c>
-      <x:c r="K14" s="11" t="str">
-        <x:v>Abarrotes</x:v>
-      </x:c>
+        <x:v>Productos Elaborados</x:v>
+      </x:c>
+      <x:c r="K14" s="11"/>
       <x:c r="L14" s="10" t="str">
-        <x:v>¿Este producto tiene un ID GetJusto vigente? Si existe, ¿cuál? Si no, confirmar que queda sin ID.</x:v>
-      </x:c>
-      <x:c r="M14" s="13" t="str"/>
+        <x:v>¿Tiene un ID GetJusto vigente? Si existe, ¿cuál? Si no, confirmar que esta fila queda sin ID.</x:v>
+      </x:c>
+      <x:c r="M14" s="13"/>
       <x:c r="N14" s="15" t="str">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="O14" s="2" t="str"/>
-      <x:c r="P14" s="14" t="str">
-        <x:v>También figura en Principal, fila 27; resolver el ID una sola vez.</x:v>
-      </x:c>
+        <x:v>232</x:v>
+      </x:c>
+      <x:c r="O14" s="2"/>
+      <x:c r="P14" s="14"/>
     </x:row>
     <x:row r="15" ht="62" customHeight="1">
       <x:c r="A15" s="2" t="str">
@@ -5579,40 +5579,40 @@
         <x:v>ID GetJusto</x:v>
       </x:c>
       <x:c r="C15" s="10" t="str">
-        <x:v>Matcha</x:v>
+        <x:v>Helado frutilla</x:v>
       </x:c>
       <x:c r="D15" s="10" t="str">
         <x:v>Barra</x:v>
       </x:c>
-      <x:c r="E15" s="10" t="str"/>
+      <x:c r="E15" s="10"/>
       <x:c r="F15" s="13" t="str">
-        <x:v>gr</x:v>
+        <x:v>Lt</x:v>
       </x:c>
       <x:c r="G15" s="16" t="str">
-        <x:v>KG</x:v>
+        <x:v>LT</x:v>
       </x:c>
       <x:c r="H15" s="13" t="str">
-        <x:v>GR ÷ 1000 = KG</x:v>
+        <x:v>1:1</x:v>
       </x:c>
       <x:c r="I15" s="13" t="str">
         <x:v>Conserva el ID GetJusto vacío y vincula por hoja y fila.</x:v>
       </x:c>
       <x:c r="J15" s="10" t="str">
-        <x:v>Te / Infusiones</x:v>
+        <x:v>Congelados</x:v>
       </x:c>
       <x:c r="K15" s="11" t="str">
-        <x:v>Cafetería</x:v>
+        <x:v>Abarrotes</x:v>
       </x:c>
       <x:c r="L15" s="10" t="str">
         <x:v>¿Este producto tiene un ID GetJusto vigente? Si existe, ¿cuál? Si no, confirmar que queda sin ID.</x:v>
       </x:c>
-      <x:c r="M15" s="13" t="str"/>
+      <x:c r="M15" s="13"/>
       <x:c r="N15" s="15" t="str">
-        <x:v>79</x:v>
-      </x:c>
-      <x:c r="O15" s="2" t="str"/>
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="O15" s="2"/>
       <x:c r="P15" s="14" t="str">
-        <x:v>También figura en Principal, fila 130; resolver el ID una sola vez.</x:v>
+        <x:v>También figura en Principal, fila 27; resolver el ID una sola vez.</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="62" customHeight="1">
@@ -5623,38 +5623,40 @@
         <x:v>ID GetJusto</x:v>
       </x:c>
       <x:c r="C16" s="10" t="str">
-        <x:v>Metilcelulosa</x:v>
+        <x:v>Matcha</x:v>
       </x:c>
       <x:c r="D16" s="10" t="str">
         <x:v>Barra</x:v>
       </x:c>
-      <x:c r="E16" s="10" t="str"/>
+      <x:c r="E16" s="10"/>
       <x:c r="F16" s="13" t="str">
-        <x:v>KG</x:v>
+        <x:v>gr</x:v>
       </x:c>
       <x:c r="G16" s="16" t="str">
         <x:v>KG</x:v>
       </x:c>
       <x:c r="H16" s="13" t="str">
-        <x:v>1:1</x:v>
+        <x:v>GR ÷ 1000 = KG</x:v>
       </x:c>
       <x:c r="I16" s="13" t="str">
         <x:v>Conserva el ID GetJusto vacío y vincula por hoja y fila.</x:v>
       </x:c>
       <x:c r="J16" s="10" t="str">
+        <x:v>Te / Infusiones</x:v>
+      </x:c>
+      <x:c r="K16" s="11" t="str">
         <x:v>Cafetería</x:v>
       </x:c>
-      <x:c r="K16" s="11" t="str"/>
       <x:c r="L16" s="10" t="str">
         <x:v>¿Este producto tiene un ID GetJusto vigente? Si existe, ¿cuál? Si no, confirmar que queda sin ID.</x:v>
       </x:c>
-      <x:c r="M16" s="13" t="str"/>
+      <x:c r="M16" s="13"/>
       <x:c r="N16" s="15" t="str">
-        <x:v>80</x:v>
-      </x:c>
-      <x:c r="O16" s="2" t="str"/>
+        <x:v>79</x:v>
+      </x:c>
+      <x:c r="O16" s="2"/>
       <x:c r="P16" s="14" t="str">
-        <x:v>También figura en Principal, fila 131; resolver el ID una sola vez.</x:v>
+        <x:v>También figura en Principal, fila 130; resolver el ID una sola vez.</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="62" customHeight="1">
@@ -5665,17 +5667,17 @@
         <x:v>ID GetJusto</x:v>
       </x:c>
       <x:c r="C17" s="10" t="str">
-        <x:v>Tenedor madera</x:v>
+        <x:v>Metilcelulosa</x:v>
       </x:c>
       <x:c r="D17" s="10" t="str">
-        <x:v>Armado / Línea / Copería</x:v>
-      </x:c>
-      <x:c r="E17" s="10" t="str"/>
+        <x:v>Barra</x:v>
+      </x:c>
+      <x:c r="E17" s="10"/>
       <x:c r="F17" s="13" t="str">
-        <x:v>UN</x:v>
+        <x:v>KG</x:v>
       </x:c>
       <x:c r="G17" s="16" t="str">
-        <x:v>UN</x:v>
+        <x:v>KG</x:v>
       </x:c>
       <x:c r="H17" s="13" t="str">
         <x:v>1:1</x:v>
@@ -5684,19 +5686,19 @@
         <x:v>Conserva el ID GetJusto vacío y vincula por hoja y fila.</x:v>
       </x:c>
       <x:c r="J17" s="10" t="str">
-        <x:v>Desechables</x:v>
-      </x:c>
-      <x:c r="K17" s="11" t="str"/>
+        <x:v>Insumos</x:v>
+      </x:c>
+      <x:c r="K17" s="11"/>
       <x:c r="L17" s="10" t="str">
         <x:v>¿Este producto tiene un ID GetJusto vigente? Si existe, ¿cuál? Si no, confirmar que queda sin ID.</x:v>
       </x:c>
-      <x:c r="M17" s="13" t="str"/>
+      <x:c r="M17" s="13"/>
       <x:c r="N17" s="15" t="str">
-        <x:v>134</x:v>
-      </x:c>
-      <x:c r="O17" s="2" t="str"/>
+        <x:v>80</x:v>
+      </x:c>
+      <x:c r="O17" s="2"/>
       <x:c r="P17" s="14" t="str">
-        <x:v>También figura en Principal, fila 213; resolver el ID una sola vez.</x:v>
+        <x:v>También figura en Principal, fila 131; resolver el ID una sola vez.</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="62" customHeight="1">
@@ -5707,12 +5709,12 @@
         <x:v>ID GetJusto</x:v>
       </x:c>
       <x:c r="C18" s="10" t="str">
-        <x:v>Cuchillo madera</x:v>
+        <x:v>Tenedor madera</x:v>
       </x:c>
       <x:c r="D18" s="10" t="str">
         <x:v>Armado / Línea / Copería</x:v>
       </x:c>
-      <x:c r="E18" s="10" t="str"/>
+      <x:c r="E18" s="10"/>
       <x:c r="F18" s="13" t="str">
         <x:v>UN</x:v>
       </x:c>
@@ -5728,17 +5730,17 @@
       <x:c r="J18" s="10" t="str">
         <x:v>Desechables</x:v>
       </x:c>
-      <x:c r="K18" s="11" t="str"/>
+      <x:c r="K18" s="11"/>
       <x:c r="L18" s="10" t="str">
         <x:v>¿Este producto tiene un ID GetJusto vigente? Si existe, ¿cuál? Si no, confirmar que queda sin ID.</x:v>
       </x:c>
-      <x:c r="M18" s="13" t="str"/>
+      <x:c r="M18" s="13"/>
       <x:c r="N18" s="15" t="str">
-        <x:v>135</x:v>
-      </x:c>
-      <x:c r="O18" s="2" t="str"/>
+        <x:v>134</x:v>
+      </x:c>
+      <x:c r="O18" s="2"/>
       <x:c r="P18" s="14" t="str">
-        <x:v>También figura en Principal, fila 214; resolver el ID una sola vez.</x:v>
+        <x:v>También figura en Principal, fila 213; resolver el ID una sola vez.</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="62" customHeight="1">
@@ -5749,12 +5751,12 @@
         <x:v>ID GetJusto</x:v>
       </x:c>
       <x:c r="C19" s="10" t="str">
-        <x:v>Cuchara madera</x:v>
+        <x:v>Cuchillo madera</x:v>
       </x:c>
       <x:c r="D19" s="10" t="str">
         <x:v>Armado / Línea / Copería</x:v>
       </x:c>
-      <x:c r="E19" s="10" t="str"/>
+      <x:c r="E19" s="10"/>
       <x:c r="F19" s="13" t="str">
         <x:v>UN</x:v>
       </x:c>
@@ -5770,17 +5772,17 @@
       <x:c r="J19" s="10" t="str">
         <x:v>Desechables</x:v>
       </x:c>
-      <x:c r="K19" s="11" t="str"/>
+      <x:c r="K19" s="11"/>
       <x:c r="L19" s="10" t="str">
         <x:v>¿Este producto tiene un ID GetJusto vigente? Si existe, ¿cuál? Si no, confirmar que queda sin ID.</x:v>
       </x:c>
-      <x:c r="M19" s="13" t="str"/>
+      <x:c r="M19" s="13"/>
       <x:c r="N19" s="15" t="str">
-        <x:v>136</x:v>
-      </x:c>
-      <x:c r="O19" s="2" t="str"/>
+        <x:v>135</x:v>
+      </x:c>
+      <x:c r="O19" s="2"/>
       <x:c r="P19" s="14" t="str">
-        <x:v>También figura en Principal, fila 215; resolver el ID una sola vez.</x:v>
+        <x:v>También figura en Principal, fila 214; resolver el ID una sola vez.</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="62" customHeight="1">
@@ -5791,40 +5793,38 @@
         <x:v>ID GetJusto</x:v>
       </x:c>
       <x:c r="C20" s="10" t="str">
-        <x:v>flor jamaica</x:v>
+        <x:v>Cuchara madera</x:v>
       </x:c>
       <x:c r="D20" s="10" t="str">
-        <x:v>Barra</x:v>
-      </x:c>
-      <x:c r="E20" s="10" t="str"/>
+        <x:v>Armado / Línea / Copería</x:v>
+      </x:c>
+      <x:c r="E20" s="10"/>
       <x:c r="F20" s="13" t="str">
-        <x:v>gr</x:v>
+        <x:v>UN</x:v>
       </x:c>
       <x:c r="G20" s="16" t="str">
-        <x:v>KG</x:v>
+        <x:v>UN</x:v>
       </x:c>
       <x:c r="H20" s="13" t="str">
-        <x:v>GR ÷ 1000 = KG</x:v>
+        <x:v>1:1</x:v>
       </x:c>
       <x:c r="I20" s="13" t="str">
         <x:v>Conserva el ID GetJusto vacío y vincula por hoja y fila.</x:v>
       </x:c>
       <x:c r="J20" s="10" t="str">
-        <x:v>Te / Infusiones</x:v>
-      </x:c>
-      <x:c r="K20" s="11" t="str">
-        <x:v>Té</x:v>
-      </x:c>
+        <x:v>Desechables</x:v>
+      </x:c>
+      <x:c r="K20" s="11"/>
       <x:c r="L20" s="10" t="str">
         <x:v>¿Este producto tiene un ID GetJusto vigente? Si existe, ¿cuál? Si no, confirmar que queda sin ID.</x:v>
       </x:c>
-      <x:c r="M20" s="13" t="str"/>
+      <x:c r="M20" s="13"/>
       <x:c r="N20" s="15" t="str">
-        <x:v>287</x:v>
-      </x:c>
-      <x:c r="O20" s="2" t="str"/>
+        <x:v>136</x:v>
+      </x:c>
+      <x:c r="O20" s="2"/>
       <x:c r="P20" s="14" t="str">
-        <x:v>También figura en Principal, fila 277; resolver el ID una sola vez.</x:v>
+        <x:v>También figura en Principal, fila 215; resolver el ID una sola vez.</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="62" customHeight="1">
@@ -5835,12 +5835,12 @@
         <x:v>ID GetJusto</x:v>
       </x:c>
       <x:c r="C21" s="10" t="str">
-        <x:v>te mariposa </x:v>
+        <x:v>flor jamaica</x:v>
       </x:c>
       <x:c r="D21" s="10" t="str">
         <x:v>Barra</x:v>
       </x:c>
-      <x:c r="E21" s="10" t="str"/>
+      <x:c r="E21" s="10"/>
       <x:c r="F21" s="13" t="str">
         <x:v>gr</x:v>
       </x:c>
@@ -5862,13 +5862,13 @@
       <x:c r="L21" s="10" t="str">
         <x:v>¿Este producto tiene un ID GetJusto vigente? Si existe, ¿cuál? Si no, confirmar que queda sin ID.</x:v>
       </x:c>
-      <x:c r="M21" s="13" t="str"/>
+      <x:c r="M21" s="13"/>
       <x:c r="N21" s="15" t="str">
-        <x:v>289</x:v>
-      </x:c>
-      <x:c r="O21" s="2" t="str"/>
+        <x:v>287</x:v>
+      </x:c>
+      <x:c r="O21" s="2"/>
       <x:c r="P21" s="14" t="str">
-        <x:v>También figura en Principal, fila 279; resolver el ID una sola vez.</x:v>
+        <x:v>También figura en Principal, fila 277; resolver el ID una sola vez.</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="62" customHeight="1">
@@ -5876,34 +5876,44 @@
         <x:v>Pendiente</x:v>
       </x:c>
       <x:c r="B22" s="2" t="str">
-        <x:v>Vínculo al Excel</x:v>
+        <x:v>ID GetJusto</x:v>
       </x:c>
       <x:c r="C22" s="10" t="str">
-        <x:v>Café Descafeinado (capsulas)</x:v>
+        <x:v>te mariposa </x:v>
       </x:c>
       <x:c r="D22" s="10" t="str">
         <x:v>Barra</x:v>
       </x:c>
-      <x:c r="E22" s="10" t="str"/>
+      <x:c r="E22" s="10"/>
       <x:c r="F22" s="13" t="str">
-        <x:v>UN</x:v>
-      </x:c>
-      <x:c r="G22" s="16" t="str"/>
-      <x:c r="H22" s="13" t="str"/>
+        <x:v>gr</x:v>
+      </x:c>
+      <x:c r="G22" s="16" t="str">
+        <x:v>KG</x:v>
+      </x:c>
+      <x:c r="H22" s="13" t="str">
+        <x:v>GR ÷ 1000 = KG</x:v>
+      </x:c>
       <x:c r="I22" s="13" t="str">
-        <x:v>Ítem heredado de Barra; vínculo de exportación pendiente. Actualmente inactivo en la app.</x:v>
+        <x:v>Conserva el ID GetJusto vacío y vincula por hoja y fila.</x:v>
       </x:c>
       <x:c r="J22" s="10" t="str">
-        <x:v>Por vincular al Excel</x:v>
-      </x:c>
-      <x:c r="K22" s="11" t="str"/>
+        <x:v>Te / Infusiones</x:v>
+      </x:c>
+      <x:c r="K22" s="11" t="str">
+        <x:v>Té</x:v>
+      </x:c>
       <x:c r="L22" s="10" t="str">
-        <x:v>Está inactivo en la app. ¿Se volverá a contar en Barra? Si sí, ¿equivale a “Café Descafeinado 504 (caja)” (fila 73) o necesita otra fila?</x:v>
-      </x:c>
-      <x:c r="M22" s="13" t="str"/>
-      <x:c r="N22" s="15" t="str"/>
-      <x:c r="O22" s="2" t="str"/>
-      <x:c r="P22" s="14" t="str"/>
+        <x:v>¿Este producto tiene un ID GetJusto vigente? Si existe, ¿cuál? Si no, confirmar que queda sin ID.</x:v>
+      </x:c>
+      <x:c r="M22" s="13"/>
+      <x:c r="N22" s="15" t="str">
+        <x:v>289</x:v>
+      </x:c>
+      <x:c r="O22" s="2"/>
+      <x:c r="P22" s="14" t="str">
+        <x:v>También figura en Principal, fila 279; resolver el ID una sola vez.</x:v>
+      </x:c>
     </x:row>
     <x:row r="23" ht="62" customHeight="1">
       <x:c r="A23" s="2" t="str">
@@ -5913,31 +5923,31 @@
         <x:v>Vínculo al Excel</x:v>
       </x:c>
       <x:c r="C23" s="10" t="str">
-        <x:v>Café descafeinado Kg</x:v>
+        <x:v>Café Descafeinado (capsulas)</x:v>
       </x:c>
       <x:c r="D23" s="10" t="str">
         <x:v>Barra</x:v>
       </x:c>
-      <x:c r="E23" s="10" t="str"/>
+      <x:c r="E23" s="10"/>
       <x:c r="F23" s="13" t="str">
-        <x:v>Kg</x:v>
-      </x:c>
-      <x:c r="G23" s="16" t="str"/>
-      <x:c r="H23" s="13" t="str"/>
+        <x:v>UN</x:v>
+      </x:c>
+      <x:c r="G23" s="16"/>
+      <x:c r="H23" s="13"/>
       <x:c r="I23" s="13" t="str">
-        <x:v>Ítem heredado de Barra; vínculo de exportación pendiente.</x:v>
+        <x:v>Ítem heredado de Barra; vínculo de exportación pendiente. Actualmente inactivo en la app.</x:v>
       </x:c>
       <x:c r="J23" s="10" t="str">
-        <x:v>Por vincular al Excel</x:v>
-      </x:c>
-      <x:c r="K23" s="11" t="str"/>
+        <x:v>Insumos</x:v>
+      </x:c>
+      <x:c r="K23" s="11"/>
       <x:c r="L23" s="10" t="str">
-        <x:v>¿Es el mismo producto que “Café Descafeinado 504 (caja)” (fila 73)? Si coincide, ¿cuántos KG equivalen a 1 UN del Excel? Si no coincide, ¿qué fila lo representa en el Excel final?</x:v>
-      </x:c>
-      <x:c r="M23" s="13" t="str"/>
-      <x:c r="N23" s="15" t="str"/>
-      <x:c r="O23" s="2" t="str"/>
-      <x:c r="P23" s="14" t="str"/>
+        <x:v>Está inactivo en la app. ¿Se volverá a contar en Barra? Si sí, ¿equivale a “Café Descafeinado 504 (caja)” (fila 73) o necesita otra fila?</x:v>
+      </x:c>
+      <x:c r="M23" s="13"/>
+      <x:c r="N23" s="15"/>
+      <x:c r="O23" s="2"/>
+      <x:c r="P23" s="14"/>
     </x:row>
     <x:row r="24" ht="62" customHeight="1">
       <x:c r="A24" s="2" t="str">
@@ -5947,31 +5957,31 @@
         <x:v>Vínculo al Excel</x:v>
       </x:c>
       <x:c r="C24" s="10" t="str">
-        <x:v>Salsa de caramelo</x:v>
+        <x:v>Café descafeinado Kg</x:v>
       </x:c>
       <x:c r="D24" s="10" t="str">
         <x:v>Barra</x:v>
       </x:c>
-      <x:c r="E24" s="10" t="str"/>
+      <x:c r="E24" s="10"/>
       <x:c r="F24" s="13" t="str">
         <x:v>Kg</x:v>
       </x:c>
-      <x:c r="G24" s="16" t="str"/>
-      <x:c r="H24" s="13" t="str"/>
+      <x:c r="G24" s="16"/>
+      <x:c r="H24" s="13"/>
       <x:c r="I24" s="13" t="str">
         <x:v>Ítem heredado de Barra; vínculo de exportación pendiente.</x:v>
       </x:c>
       <x:c r="J24" s="10" t="str">
-        <x:v>Por vincular al Excel</x:v>
-      </x:c>
-      <x:c r="K24" s="11" t="str"/>
+        <x:v>Insumos</x:v>
+      </x:c>
+      <x:c r="K24" s="11"/>
       <x:c r="L24" s="10" t="str">
-        <x:v>¿Es el mismo producto que “Salsa caramelo” (fila 152)? Si coincide, ¿cuántos KG equivalen a 1 UN del Excel? Si no coincide, ¿qué fila lo representa en el Excel final?</x:v>
-      </x:c>
-      <x:c r="M24" s="13" t="str"/>
-      <x:c r="N24" s="15" t="str"/>
-      <x:c r="O24" s="2" t="str"/>
-      <x:c r="P24" s="14" t="str"/>
+        <x:v>¿Es el mismo producto que “Café Descafeinado 504 (caja)” (fila 73)? Si coincide, ¿cuántos KG equivalen a 1 UN del Excel? Si no coincide, ¿qué fila lo representa en el Excel final?</x:v>
+      </x:c>
+      <x:c r="M24" s="13"/>
+      <x:c r="N24" s="15"/>
+      <x:c r="O24" s="2"/>
+      <x:c r="P24" s="14"/>
     </x:row>
     <x:row r="25" ht="62" customHeight="1">
       <x:c r="A25" s="2" t="str">
@@ -5981,31 +5991,31 @@
         <x:v>Vínculo al Excel</x:v>
       </x:c>
       <x:c r="C25" s="10" t="str">
-        <x:v>Metafisulfito de sodio</x:v>
+        <x:v>Salsa de caramelo</x:v>
       </x:c>
       <x:c r="D25" s="10" t="str">
         <x:v>Barra</x:v>
       </x:c>
-      <x:c r="E25" s="10" t="str"/>
+      <x:c r="E25" s="10"/>
       <x:c r="F25" s="13" t="str">
-        <x:v>gr</x:v>
-      </x:c>
-      <x:c r="G25" s="16" t="str"/>
-      <x:c r="H25" s="13" t="str"/>
+        <x:v>Kg</x:v>
+      </x:c>
+      <x:c r="G25" s="16"/>
+      <x:c r="H25" s="13"/>
       <x:c r="I25" s="13" t="str">
         <x:v>Ítem heredado de Barra; vínculo de exportación pendiente.</x:v>
       </x:c>
       <x:c r="J25" s="10" t="str">
-        <x:v>Por vincular al Excel</x:v>
-      </x:c>
-      <x:c r="K25" s="11" t="str"/>
+        <x:v>Insumos</x:v>
+      </x:c>
+      <x:c r="K25" s="11"/>
       <x:c r="L25" s="10" t="str">
-        <x:v>¿Se usa y cuenta hoy en Barra? ¿Es el mismo metabisulfito de sodio que aparece en otras áreas? No hay fila de este producto en Servicio.</x:v>
-      </x:c>
-      <x:c r="M25" s="13" t="str"/>
-      <x:c r="N25" s="15" t="str"/>
-      <x:c r="O25" s="2" t="str"/>
-      <x:c r="P25" s="14" t="str"/>
+        <x:v>¿Es el mismo producto que “Salsa caramelo” (fila 152)? Si coincide, ¿cuántos KG equivalen a 1 UN del Excel? Si no coincide, ¿qué fila lo representa en el Excel final?</x:v>
+      </x:c>
+      <x:c r="M25" s="13"/>
+      <x:c r="N25" s="15"/>
+      <x:c r="O25" s="2"/>
+      <x:c r="P25" s="14"/>
     </x:row>
     <x:row r="26" ht="62" customHeight="1">
       <x:c r="A26" s="2" t="str">
@@ -6015,31 +6025,31 @@
         <x:v>Vínculo al Excel</x:v>
       </x:c>
       <x:c r="C26" s="10" t="str">
-        <x:v>PE PORCION JUGO NARANJA (EXTRA)</x:v>
+        <x:v>Metafisulfito de sodio</x:v>
       </x:c>
       <x:c r="D26" s="10" t="str">
         <x:v>Barra</x:v>
       </x:c>
-      <x:c r="E26" s="10" t="str"/>
+      <x:c r="E26" s="10"/>
       <x:c r="F26" s="13" t="str">
-        <x:v>UN</x:v>
-      </x:c>
-      <x:c r="G26" s="16" t="str"/>
-      <x:c r="H26" s="13" t="str"/>
+        <x:v>gr</x:v>
+      </x:c>
+      <x:c r="G26" s="16"/>
+      <x:c r="H26" s="13"/>
       <x:c r="I26" s="13" t="str">
         <x:v>Ítem heredado de Barra; vínculo de exportación pendiente.</x:v>
       </x:c>
       <x:c r="J26" s="10" t="str">
-        <x:v>Por vincular al Excel</x:v>
-      </x:c>
-      <x:c r="K26" s="11" t="str"/>
+        <x:v>Insumos</x:v>
+      </x:c>
+      <x:c r="K26" s="11"/>
       <x:c r="L26" s="10" t="str">
-        <x:v>Ya se aclaró que esta porción es un producto nuevo sin fila en el totalizado. ¿Se sigue contando en Barra y cómo se tratará al exportar mientras falte una fila oficial?</x:v>
-      </x:c>
-      <x:c r="M26" s="13" t="str"/>
-      <x:c r="N26" s="15" t="str"/>
-      <x:c r="O26" s="2" t="str"/>
-      <x:c r="P26" s="14" t="str"/>
+        <x:v>¿Se usa y cuenta hoy en Barra? ¿Es el mismo metabisulfito de sodio que aparece en otras áreas? No hay fila de este producto en Servicio.</x:v>
+      </x:c>
+      <x:c r="M26" s="13"/>
+      <x:c r="N26" s="15"/>
+      <x:c r="O26" s="2"/>
+      <x:c r="P26" s="14"/>
     </x:row>
     <x:row r="27" ht="62" customHeight="1">
       <x:c r="A27" s="2" t="str">
@@ -6049,31 +6059,31 @@
         <x:v>Vínculo al Excel</x:v>
       </x:c>
       <x:c r="C27" s="10" t="str">
-        <x:v>PE PORCION JUGO PRIMAVERAL (EXTRA)</x:v>
+        <x:v>PE PORCION JUGO NARANJA (EXTRA)</x:v>
       </x:c>
       <x:c r="D27" s="10" t="str">
         <x:v>Barra</x:v>
       </x:c>
-      <x:c r="E27" s="10" t="str"/>
+      <x:c r="E27" s="10"/>
       <x:c r="F27" s="13" t="str">
         <x:v>UN</x:v>
       </x:c>
-      <x:c r="G27" s="16" t="str"/>
-      <x:c r="H27" s="13" t="str"/>
+      <x:c r="G27" s="16"/>
+      <x:c r="H27" s="13"/>
       <x:c r="I27" s="13" t="str">
         <x:v>Ítem heredado de Barra; vínculo de exportación pendiente.</x:v>
       </x:c>
       <x:c r="J27" s="10" t="str">
-        <x:v>Por vincular al Excel</x:v>
-      </x:c>
-      <x:c r="K27" s="11" t="str"/>
+        <x:v>Congelados</x:v>
+      </x:c>
+      <x:c r="K27" s="11"/>
       <x:c r="L27" s="10" t="str">
-        <x:v>¿Es el mismo producto que “Primaveral” (fila 62)? Si no coincide, ¿qué fila lo representa en el Excel final?</x:v>
-      </x:c>
-      <x:c r="M27" s="13" t="str"/>
-      <x:c r="N27" s="15" t="str"/>
-      <x:c r="O27" s="2" t="str"/>
-      <x:c r="P27" s="14" t="str"/>
+        <x:v>Ya se aclaró que esta porción es un producto nuevo sin fila en el totalizado. ¿Se sigue contando en Barra y cómo se tratará al exportar mientras falte una fila oficial?</x:v>
+      </x:c>
+      <x:c r="M27" s="13"/>
+      <x:c r="N27" s="15"/>
+      <x:c r="O27" s="2"/>
+      <x:c r="P27" s="14"/>
     </x:row>
     <x:row r="28" ht="62" customHeight="1">
       <x:c r="A28" s="2" t="str">
@@ -6083,31 +6093,31 @@
         <x:v>Vínculo al Excel</x:v>
       </x:c>
       <x:c r="C28" s="10" t="str">
-        <x:v>PE PORCION JUGO MANCORA (EXTRA)</x:v>
+        <x:v>PE PORCION JUGO PRIMAVERAL (EXTRA)</x:v>
       </x:c>
       <x:c r="D28" s="10" t="str">
         <x:v>Barra</x:v>
       </x:c>
-      <x:c r="E28" s="10" t="str"/>
+      <x:c r="E28" s="10"/>
       <x:c r="F28" s="13" t="str">
         <x:v>UN</x:v>
       </x:c>
-      <x:c r="G28" s="16" t="str"/>
-      <x:c r="H28" s="13" t="str"/>
+      <x:c r="G28" s="16"/>
+      <x:c r="H28" s="13"/>
       <x:c r="I28" s="13" t="str">
         <x:v>Ítem heredado de Barra; vínculo de exportación pendiente.</x:v>
       </x:c>
       <x:c r="J28" s="10" t="str">
-        <x:v>Por vincular al Excel</x:v>
-      </x:c>
-      <x:c r="K28" s="11" t="str"/>
+        <x:v>Congelados</x:v>
+      </x:c>
+      <x:c r="K28" s="11"/>
       <x:c r="L28" s="10" t="str">
-        <x:v>¿Se prepara o cuenta todavía esta porción? No aparece una fila equivalente en Servicio; ¿cómo se registrará al exportar?</x:v>
-      </x:c>
-      <x:c r="M28" s="13" t="str"/>
-      <x:c r="N28" s="15" t="str"/>
-      <x:c r="O28" s="2" t="str"/>
-      <x:c r="P28" s="14" t="str"/>
+        <x:v>¿Es el mismo producto que “Primaveral” (fila 62)? Si no coincide, ¿qué fila lo representa en el Excel final?</x:v>
+      </x:c>
+      <x:c r="M28" s="13"/>
+      <x:c r="N28" s="15"/>
+      <x:c r="O28" s="2"/>
+      <x:c r="P28" s="14"/>
     </x:row>
     <x:row r="29" ht="62" customHeight="1">
       <x:c r="A29" s="2" t="str">
@@ -6117,31 +6127,31 @@
         <x:v>Vínculo al Excel</x:v>
       </x:c>
       <x:c r="C29" s="10" t="str">
-        <x:v>Leche desc / sin lactosa 1 Lt</x:v>
+        <x:v>PE PORCION JUGO MANCORA (EXTRA)</x:v>
       </x:c>
       <x:c r="D29" s="10" t="str">
         <x:v>Barra</x:v>
       </x:c>
-      <x:c r="E29" s="10" t="str"/>
+      <x:c r="E29" s="10"/>
       <x:c r="F29" s="13" t="str">
-        <x:v>Lt</x:v>
-      </x:c>
-      <x:c r="G29" s="16" t="str"/>
-      <x:c r="H29" s="13" t="str"/>
+        <x:v>UN</x:v>
+      </x:c>
+      <x:c r="G29" s="16"/>
+      <x:c r="H29" s="13"/>
       <x:c r="I29" s="13" t="str">
         <x:v>Ítem heredado de Barra; vínculo de exportación pendiente.</x:v>
       </x:c>
       <x:c r="J29" s="10" t="str">
-        <x:v>Por vincular al Excel</x:v>
-      </x:c>
-      <x:c r="K29" s="11" t="str"/>
+        <x:v>Congelados</x:v>
+      </x:c>
+      <x:c r="K29" s="11"/>
       <x:c r="L29" s="10" t="str">
-        <x:v>¿Es el mismo producto que “Leche desc / sin lactosa unidad 1 lt” (fila 140)? Si no coincide, ¿qué fila lo representa en el Excel final?</x:v>
-      </x:c>
-      <x:c r="M29" s="13" t="str"/>
-      <x:c r="N29" s="15" t="str"/>
-      <x:c r="O29" s="2" t="str"/>
-      <x:c r="P29" s="14" t="str"/>
+        <x:v>¿Se prepara o cuenta todavía esta porción? No aparece una fila equivalente en Servicio; ¿cómo se registrará al exportar?</x:v>
+      </x:c>
+      <x:c r="M29" s="13"/>
+      <x:c r="N29" s="15"/>
+      <x:c r="O29" s="2"/>
+      <x:c r="P29" s="14"/>
     </x:row>
     <x:row r="30" ht="62" customHeight="1">
       <x:c r="A30" s="2" t="str">
@@ -6151,31 +6161,31 @@
         <x:v>Vínculo al Excel</x:v>
       </x:c>
       <x:c r="C30" s="10" t="str">
-        <x:v>TAPA VASO 350 CC PLASTICO</x:v>
+        <x:v>Leche desc / sin lactosa 1 Lt</x:v>
       </x:c>
       <x:c r="D30" s="10" t="str">
         <x:v>Barra</x:v>
       </x:c>
-      <x:c r="E30" s="10" t="str"/>
+      <x:c r="E30" s="10"/>
       <x:c r="F30" s="13" t="str">
-        <x:v>UN</x:v>
-      </x:c>
-      <x:c r="G30" s="16" t="str"/>
-      <x:c r="H30" s="13" t="str"/>
+        <x:v>Lt</x:v>
+      </x:c>
+      <x:c r="G30" s="16"/>
+      <x:c r="H30" s="13"/>
       <x:c r="I30" s="13" t="str">
         <x:v>Ítem heredado de Barra; vínculo de exportación pendiente.</x:v>
       </x:c>
       <x:c r="J30" s="10" t="str">
-        <x:v>Por vincular al Excel</x:v>
-      </x:c>
-      <x:c r="K30" s="11" t="str"/>
+        <x:v>Insumos</x:v>
+      </x:c>
+      <x:c r="K30" s="11"/>
       <x:c r="L30" s="10" t="str">
-        <x:v>¿Qué tapa del Excel final corresponde a este vaso de 350 cc? No hay una coincidencia clara por nombre.</x:v>
-      </x:c>
-      <x:c r="M30" s="13" t="str"/>
-      <x:c r="N30" s="15" t="str"/>
-      <x:c r="O30" s="2" t="str"/>
-      <x:c r="P30" s="14" t="str"/>
+        <x:v>¿Es el mismo producto que “Leche desc / sin lactosa unidad 1 lt” (fila 140)? Si no coincide, ¿qué fila lo representa en el Excel final?</x:v>
+      </x:c>
+      <x:c r="M30" s="13"/>
+      <x:c r="N30" s="15"/>
+      <x:c r="O30" s="2"/>
+      <x:c r="P30" s="14"/>
     </x:row>
     <x:row r="31" ht="62" customHeight="1">
       <x:c r="A31" s="2" t="str">
@@ -6185,31 +6195,31 @@
         <x:v>Vínculo al Excel</x:v>
       </x:c>
       <x:c r="C31" s="10" t="str">
-        <x:v>TAPA VASO KRAFT DE CAFÉ CHICO 8 OZ</x:v>
+        <x:v>TAPA VASO 350 CC PLASTICO</x:v>
       </x:c>
       <x:c r="D31" s="10" t="str">
         <x:v>Barra</x:v>
       </x:c>
-      <x:c r="E31" s="10" t="str"/>
+      <x:c r="E31" s="10"/>
       <x:c r="F31" s="13" t="str">
         <x:v>UN</x:v>
       </x:c>
-      <x:c r="G31" s="16" t="str"/>
-      <x:c r="H31" s="13" t="str"/>
+      <x:c r="G31" s="16"/>
+      <x:c r="H31" s="13"/>
       <x:c r="I31" s="13" t="str">
         <x:v>Ítem heredado de Barra; vínculo de exportación pendiente.</x:v>
       </x:c>
       <x:c r="J31" s="10" t="str">
-        <x:v>Por vincular al Excel</x:v>
-      </x:c>
-      <x:c r="K31" s="11" t="str"/>
+        <x:v>Desechables</x:v>
+      </x:c>
+      <x:c r="K31" s="11"/>
       <x:c r="L31" s="10" t="str">
-        <x:v>¿Es el mismo producto que “TAPA VASO KRAFT DE CAFÉ CHICO 8 OZ (10x100)” (fila 125)? Si no coincide, ¿qué fila lo representa en el Excel final?</x:v>
-      </x:c>
-      <x:c r="M31" s="13" t="str"/>
-      <x:c r="N31" s="15" t="str"/>
-      <x:c r="O31" s="2" t="str"/>
-      <x:c r="P31" s="14" t="str"/>
+        <x:v>¿Qué tapa del Excel final corresponde a este vaso de 350 cc? No hay una coincidencia clara por nombre.</x:v>
+      </x:c>
+      <x:c r="M31" s="13"/>
+      <x:c r="N31" s="15"/>
+      <x:c r="O31" s="2"/>
+      <x:c r="P31" s="14"/>
     </x:row>
     <x:row r="32" ht="62" customHeight="1">
       <x:c r="A32" s="2" t="str">
@@ -6219,31 +6229,31 @@
         <x:v>Vínculo al Excel</x:v>
       </x:c>
       <x:c r="C32" s="10" t="str">
-        <x:v>TAPA VASO KRAFT DE CAFÉ GRANDE 12/16 OZ</x:v>
+        <x:v>TAPA VASO KRAFT DE CAFÉ CHICO 8 OZ</x:v>
       </x:c>
       <x:c r="D32" s="10" t="str">
         <x:v>Barra</x:v>
       </x:c>
-      <x:c r="E32" s="10" t="str"/>
+      <x:c r="E32" s="10"/>
       <x:c r="F32" s="13" t="str">
         <x:v>UN</x:v>
       </x:c>
-      <x:c r="G32" s="16" t="str"/>
-      <x:c r="H32" s="13" t="str"/>
+      <x:c r="G32" s="16"/>
+      <x:c r="H32" s="13"/>
       <x:c r="I32" s="13" t="str">
         <x:v>Ítem heredado de Barra; vínculo de exportación pendiente.</x:v>
       </x:c>
       <x:c r="J32" s="10" t="str">
-        <x:v>Por vincular al Excel</x:v>
-      </x:c>
-      <x:c r="K32" s="11" t="str"/>
+        <x:v>Desechables</x:v>
+      </x:c>
+      <x:c r="K32" s="11"/>
       <x:c r="L32" s="10" t="str">
-        <x:v>¿Es el mismo producto que “TAPA VASO KRAFT DE CAFÉ GRANDE 12/16 OZ (20x50)” (fila 126)? Si no coincide, ¿qué fila lo representa en el Excel final?</x:v>
-      </x:c>
-      <x:c r="M32" s="13" t="str"/>
-      <x:c r="N32" s="15" t="str"/>
-      <x:c r="O32" s="2" t="str"/>
-      <x:c r="P32" s="14" t="str"/>
+        <x:v>¿Es el mismo producto que “TAPA VASO KRAFT DE CAFÉ CHICO 8 OZ (10x100)” (fila 125)? Si no coincide, ¿qué fila lo representa en el Excel final?</x:v>
+      </x:c>
+      <x:c r="M32" s="13"/>
+      <x:c r="N32" s="15"/>
+      <x:c r="O32" s="2"/>
+      <x:c r="P32" s="14"/>
     </x:row>
     <x:row r="33" ht="62" customHeight="1">
       <x:c r="A33" s="2" t="str">
@@ -6253,31 +6263,31 @@
         <x:v>Vínculo al Excel</x:v>
       </x:c>
       <x:c r="C33" s="10" t="str">
-        <x:v>VASOS 350 CC PLASTICO</x:v>
+        <x:v>TAPA VASO KRAFT DE CAFÉ GRANDE 12/16 OZ</x:v>
       </x:c>
       <x:c r="D33" s="10" t="str">
         <x:v>Barra</x:v>
       </x:c>
-      <x:c r="E33" s="10" t="str"/>
+      <x:c r="E33" s="10"/>
       <x:c r="F33" s="13" t="str">
         <x:v>UN</x:v>
       </x:c>
-      <x:c r="G33" s="16" t="str"/>
-      <x:c r="H33" s="13" t="str"/>
+      <x:c r="G33" s="16"/>
+      <x:c r="H33" s="13"/>
       <x:c r="I33" s="13" t="str">
         <x:v>Ítem heredado de Barra; vínculo de exportación pendiente.</x:v>
       </x:c>
       <x:c r="J33" s="10" t="str">
-        <x:v>Por vincular al Excel</x:v>
-      </x:c>
-      <x:c r="K33" s="11" t="str"/>
+        <x:v>Desechables</x:v>
+      </x:c>
+      <x:c r="K33" s="11"/>
       <x:c r="L33" s="10" t="str">
-        <x:v>¿Es el mismo producto que “VASOS 350 CC PLASTICO (1x2800)” (fila 131)? Si no coincide, ¿qué fila lo representa en el Excel final?</x:v>
-      </x:c>
-      <x:c r="M33" s="13" t="str"/>
-      <x:c r="N33" s="15" t="str"/>
-      <x:c r="O33" s="2" t="str"/>
-      <x:c r="P33" s="14" t="str"/>
+        <x:v>¿Es el mismo producto que “TAPA VASO KRAFT DE CAFÉ GRANDE 12/16 OZ (20x50)” (fila 126)? Si no coincide, ¿qué fila lo representa en el Excel final?</x:v>
+      </x:c>
+      <x:c r="M33" s="13"/>
+      <x:c r="N33" s="15"/>
+      <x:c r="O33" s="2"/>
+      <x:c r="P33" s="14"/>
     </x:row>
     <x:row r="34" ht="62" customHeight="1">
       <x:c r="A34" s="2" t="str">
@@ -6287,31 +6297,31 @@
         <x:v>Vínculo al Excel</x:v>
       </x:c>
       <x:c r="C34" s="10" t="str">
-        <x:v>VASOS KRAFT LA BRIOCHE CHICO 8 OZ</x:v>
+        <x:v>VASOS 350 CC PLASTICO</x:v>
       </x:c>
       <x:c r="D34" s="10" t="str">
         <x:v>Barra</x:v>
       </x:c>
-      <x:c r="E34" s="10" t="str"/>
+      <x:c r="E34" s="10"/>
       <x:c r="F34" s="13" t="str">
         <x:v>UN</x:v>
       </x:c>
-      <x:c r="G34" s="16" t="str"/>
-      <x:c r="H34" s="13" t="str"/>
+      <x:c r="G34" s="16"/>
+      <x:c r="H34" s="13"/>
       <x:c r="I34" s="13" t="str">
         <x:v>Ítem heredado de Barra; vínculo de exportación pendiente.</x:v>
       </x:c>
       <x:c r="J34" s="10" t="str">
-        <x:v>Por vincular al Excel</x:v>
-      </x:c>
-      <x:c r="K34" s="11" t="str"/>
+        <x:v>Desechables</x:v>
+      </x:c>
+      <x:c r="K34" s="11"/>
       <x:c r="L34" s="10" t="str">
-        <x:v>¿Es el mismo producto que “VASOS KRAFT LA BRIOCHE CHICO 8 OZ (20X50)” (fila 132)? Si no coincide, ¿qué fila lo representa en el Excel final?</x:v>
-      </x:c>
-      <x:c r="M34" s="13" t="str"/>
-      <x:c r="N34" s="15" t="str"/>
-      <x:c r="O34" s="2" t="str"/>
-      <x:c r="P34" s="14" t="str"/>
+        <x:v>¿Es el mismo producto que “VASOS 350 CC PLASTICO (1x2800)” (fila 131)? Si no coincide, ¿qué fila lo representa en el Excel final?</x:v>
+      </x:c>
+      <x:c r="M34" s="13"/>
+      <x:c r="N34" s="15"/>
+      <x:c r="O34" s="2"/>
+      <x:c r="P34" s="14"/>
     </x:row>
     <x:row r="35" ht="62" customHeight="1">
       <x:c r="A35" s="2" t="str">
@@ -6321,31 +6331,31 @@
         <x:v>Vínculo al Excel</x:v>
       </x:c>
       <x:c r="C35" s="10" t="str">
-        <x:v>VASOS KRAFT LA BRIOCHE MEDIANO 12 OZ</x:v>
+        <x:v>VASOS KRAFT LA BRIOCHE CHICO 8 OZ</x:v>
       </x:c>
       <x:c r="D35" s="10" t="str">
         <x:v>Barra</x:v>
       </x:c>
-      <x:c r="E35" s="10" t="str"/>
+      <x:c r="E35" s="10"/>
       <x:c r="F35" s="13" t="str">
         <x:v>UN</x:v>
       </x:c>
-      <x:c r="G35" s="16" t="str"/>
-      <x:c r="H35" s="13" t="str"/>
+      <x:c r="G35" s="16"/>
+      <x:c r="H35" s="13"/>
       <x:c r="I35" s="13" t="str">
         <x:v>Ítem heredado de Barra; vínculo de exportación pendiente.</x:v>
       </x:c>
       <x:c r="J35" s="10" t="str">
-        <x:v>Por vincular al Excel</x:v>
-      </x:c>
-      <x:c r="K35" s="11" t="str"/>
+        <x:v>Desechables</x:v>
+      </x:c>
+      <x:c r="K35" s="11"/>
       <x:c r="L35" s="10" t="str">
-        <x:v>¿Es el mismo producto que “VASOS KRAFT LA BRIOCHE MEDIANO 12 OZ (50X20)” (fila 133)? Si no coincide, ¿qué fila lo representa en el Excel final?</x:v>
-      </x:c>
-      <x:c r="M35" s="13" t="str"/>
-      <x:c r="N35" s="15" t="str"/>
-      <x:c r="O35" s="2" t="str"/>
-      <x:c r="P35" s="14" t="str"/>
+        <x:v>¿Es el mismo producto que “VASOS KRAFT LA BRIOCHE CHICO 8 OZ (20X50)” (fila 132)? Si no coincide, ¿qué fila lo representa en el Excel final?</x:v>
+      </x:c>
+      <x:c r="M35" s="13"/>
+      <x:c r="N35" s="15"/>
+      <x:c r="O35" s="2"/>
+      <x:c r="P35" s="14"/>
     </x:row>
     <x:row r="36" ht="62" customHeight="1">
       <x:c r="A36" s="2" t="str">
@@ -6355,31 +6365,31 @@
         <x:v>Vínculo al Excel</x:v>
       </x:c>
       <x:c r="C36" s="10" t="str">
-        <x:v>Bicarbonato</x:v>
+        <x:v>VASOS KRAFT LA BRIOCHE MEDIANO 12 OZ</x:v>
       </x:c>
       <x:c r="D36" s="10" t="str">
         <x:v>Barra</x:v>
       </x:c>
-      <x:c r="E36" s="10" t="str"/>
+      <x:c r="E36" s="10"/>
       <x:c r="F36" s="13" t="str">
-        <x:v>gr</x:v>
-      </x:c>
-      <x:c r="G36" s="16" t="str"/>
-      <x:c r="H36" s="13" t="str"/>
+        <x:v>UN</x:v>
+      </x:c>
+      <x:c r="G36" s="16"/>
+      <x:c r="H36" s="13"/>
       <x:c r="I36" s="13" t="str">
         <x:v>Ítem heredado de Barra; vínculo de exportación pendiente.</x:v>
       </x:c>
       <x:c r="J36" s="10" t="str">
-        <x:v>Por vincular al Excel</x:v>
-      </x:c>
-      <x:c r="K36" s="11" t="str"/>
+        <x:v>Desechables</x:v>
+      </x:c>
+      <x:c r="K36" s="11"/>
       <x:c r="L36" s="10" t="str">
-        <x:v>¿Es el mismo producto que “Bicarbonato kg” (fila 145)? Si no coincide, ¿qué fila lo representa en el Excel final?</x:v>
-      </x:c>
-      <x:c r="M36" s="13" t="str"/>
-      <x:c r="N36" s="15" t="str"/>
-      <x:c r="O36" s="2" t="str"/>
-      <x:c r="P36" s="14" t="str"/>
+        <x:v>¿Es el mismo producto que “VASOS KRAFT LA BRIOCHE MEDIANO 12 OZ (50X20)” (fila 133)? Si no coincide, ¿qué fila lo representa en el Excel final?</x:v>
+      </x:c>
+      <x:c r="M36" s="13"/>
+      <x:c r="N36" s="15"/>
+      <x:c r="O36" s="2"/>
+      <x:c r="P36" s="14"/>
     </x:row>
     <x:row r="37" ht="62" customHeight="1">
       <x:c r="A37" s="2" t="str">
@@ -6389,31 +6399,31 @@
         <x:v>Vínculo al Excel</x:v>
       </x:c>
       <x:c r="C37" s="10" t="str">
-        <x:v>Fruta congelada Arándano</x:v>
+        <x:v>Bicarbonato</x:v>
       </x:c>
       <x:c r="D37" s="10" t="str">
         <x:v>Barra</x:v>
       </x:c>
-      <x:c r="E37" s="10" t="str"/>
+      <x:c r="E37" s="10"/>
       <x:c r="F37" s="13" t="str">
-        <x:v>Kg</x:v>
-      </x:c>
-      <x:c r="G37" s="16" t="str"/>
-      <x:c r="H37" s="13" t="str"/>
+        <x:v>gr</x:v>
+      </x:c>
+      <x:c r="G37" s="16"/>
+      <x:c r="H37" s="13"/>
       <x:c r="I37" s="13" t="str">
         <x:v>Ítem heredado de Barra; vínculo de exportación pendiente.</x:v>
       </x:c>
       <x:c r="J37" s="10" t="str">
-        <x:v>Por vincular al Excel</x:v>
-      </x:c>
-      <x:c r="K37" s="11" t="str"/>
+        <x:v>Limpieza</x:v>
+      </x:c>
+      <x:c r="K37" s="11"/>
       <x:c r="L37" s="10" t="str">
-        <x:v>¿Barra guarda y cuenta arándanos congelados? Hay una fila en Bodega, pero no en Servicio; ¿cómo se reflejará el stock de Barra?</x:v>
-      </x:c>
-      <x:c r="M37" s="13" t="str"/>
-      <x:c r="N37" s="15" t="str"/>
-      <x:c r="O37" s="2" t="str"/>
-      <x:c r="P37" s="14" t="str"/>
+        <x:v>¿Es el mismo producto que “Bicarbonato kg” (fila 145)? Si no coincide, ¿qué fila lo representa en el Excel final?</x:v>
+      </x:c>
+      <x:c r="M37" s="13"/>
+      <x:c r="N37" s="15"/>
+      <x:c r="O37" s="2"/>
+      <x:c r="P37" s="14"/>
     </x:row>
     <x:row r="38" ht="62" customHeight="1">
       <x:c r="A38" s="2" t="str">
@@ -6423,31 +6433,31 @@
         <x:v>Vínculo al Excel</x:v>
       </x:c>
       <x:c r="C38" s="10" t="str">
-        <x:v>Crema Vegetal</x:v>
+        <x:v>Fruta congelada Arándano</x:v>
       </x:c>
       <x:c r="D38" s="10" t="str">
         <x:v>Barra</x:v>
       </x:c>
-      <x:c r="E38" s="10" t="str"/>
+      <x:c r="E38" s="10"/>
       <x:c r="F38" s="13" t="str">
-        <x:v>Lt</x:v>
-      </x:c>
-      <x:c r="G38" s="16" t="str"/>
-      <x:c r="H38" s="13" t="str"/>
+        <x:v>Kg</x:v>
+      </x:c>
+      <x:c r="G38" s="16"/>
+      <x:c r="H38" s="13"/>
       <x:c r="I38" s="13" t="str">
         <x:v>Ítem heredado de Barra; vínculo de exportación pendiente.</x:v>
       </x:c>
       <x:c r="J38" s="10" t="str">
-        <x:v>Por vincular al Excel</x:v>
-      </x:c>
-      <x:c r="K38" s="11" t="str"/>
+        <x:v>Congelados</x:v>
+      </x:c>
+      <x:c r="K38" s="11"/>
       <x:c r="L38" s="10" t="str">
-        <x:v>¿Es el mismo producto que “Crema Vegetal MONA LISA” (fila 139)? Si no coincide, ¿qué fila lo representa en el Excel final?</x:v>
-      </x:c>
-      <x:c r="M38" s="13" t="str"/>
-      <x:c r="N38" s="15" t="str"/>
-      <x:c r="O38" s="2" t="str"/>
-      <x:c r="P38" s="14" t="str"/>
+        <x:v>¿Barra guarda y cuenta arándanos congelados? Hay una fila en Bodega, pero no en Servicio; ¿cómo se reflejará el stock de Barra?</x:v>
+      </x:c>
+      <x:c r="M38" s="13"/>
+      <x:c r="N38" s="15"/>
+      <x:c r="O38" s="2"/>
+      <x:c r="P38" s="14"/>
     </x:row>
     <x:row r="39" ht="62" customHeight="1">
       <x:c r="A39" s="2" t="str">
@@ -6457,46 +6467,62 @@
         <x:v>Vínculo al Excel</x:v>
       </x:c>
       <x:c r="C39" s="10" t="str">
-        <x:v>Frutillas congeladas</x:v>
+        <x:v>Crema Vegetal</x:v>
       </x:c>
       <x:c r="D39" s="10" t="str">
         <x:v>Barra</x:v>
       </x:c>
-      <x:c r="E39" s="10" t="str"/>
+      <x:c r="E39" s="10"/>
       <x:c r="F39" s="13" t="str">
-        <x:v>Kg</x:v>
-      </x:c>
-      <x:c r="G39" s="16" t="str"/>
-      <x:c r="H39" s="13" t="str"/>
+        <x:v>Lt</x:v>
+      </x:c>
+      <x:c r="G39" s="16"/>
+      <x:c r="H39" s="13"/>
       <x:c r="I39" s="13" t="str">
         <x:v>Ítem heredado de Barra; vínculo de exportación pendiente.</x:v>
       </x:c>
       <x:c r="J39" s="10" t="str">
-        <x:v>Por vincular al Excel</x:v>
-      </x:c>
-      <x:c r="K39" s="11" t="str"/>
+        <x:v>Insumos</x:v>
+      </x:c>
+      <x:c r="K39" s="11"/>
       <x:c r="L39" s="10" t="str">
+        <x:v>¿Es el mismo producto que “Crema Vegetal MONA LISA” (fila 139)? Si no coincide, ¿qué fila lo representa en el Excel final?</x:v>
+      </x:c>
+      <x:c r="M39" s="13"/>
+      <x:c r="N39" s="15"/>
+      <x:c r="O39" s="2"/>
+      <x:c r="P39" s="14"/>
+    </x:row>
+    <x:row r="40" ht="62" customHeight="1">
+      <x:c r="A40" s="2" t="str">
+        <x:v>Pendiente</x:v>
+      </x:c>
+      <x:c r="B40" s="2" t="str">
+        <x:v>Vínculo al Excel</x:v>
+      </x:c>
+      <x:c r="C40" s="10" t="str">
+        <x:v>Frutillas congeladas</x:v>
+      </x:c>
+      <x:c r="D40" s="10" t="str">
+        <x:v>Barra</x:v>
+      </x:c>
+      <x:c r="E40" s="10"/>
+      <x:c r="F40" s="13" t="str">
+        <x:v>Kg</x:v>
+      </x:c>
+      <x:c r="G40" s="16"/>
+      <x:c r="H40" s="13"/>
+      <x:c r="I40" s="13" t="str">
+        <x:v>Ítem heredado de Barra; vínculo de exportación pendiente.</x:v>
+      </x:c>
+      <x:c r="J40" s="10" t="str">
+        <x:v>Congelados</x:v>
+      </x:c>
+      <x:c r="K40" s="11"/>
+      <x:c r="L40" s="10" t="str">
         <x:v>¿Es el mismo producto que “Frutillas” (fila 137)? Si no coincide, ¿qué fila lo representa en el Excel final?</x:v>
       </x:c>
-      <x:c r="M39" s="13" t="str"/>
-      <x:c r="N39" s="15" t="str"/>
-      <x:c r="O39" s="2" t="str"/>
-      <x:c r="P39" s="14" t="str"/>
-    </x:row>
-    <x:row r="40" ht="37" customHeight="1">
-      <x:c r="A40" s="2"/>
-      <x:c r="B40" s="2"/>
-      <x:c r="C40" s="2"/>
-      <x:c r="D40" s="2"/>
-      <x:c r="E40" s="2"/>
-      <x:c r="F40" s="14"/>
-      <x:c r="G40" s="15"/>
-      <x:c r="H40" s="14"/>
-      <x:c r="I40" s="14"/>
-      <x:c r="J40" s="2"/>
-      <x:c r="K40" s="12"/>
-      <x:c r="L40" s="2"/>
-      <x:c r="M40" s="14"/>
+      <x:c r="M40" s="13"/>
       <x:c r="N40" s="15"/>
       <x:c r="O40" s="2"/>
       <x:c r="P40" s="14"/>
@@ -6933,7 +6959,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1afbc6ace7b44253"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4b5c4e670da240dd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7094,7 +7120,7 @@
         <x:v>Hoy muestra y guarda KG; factor configurado 1:1.</x:v>
       </x:c>
       <x:c r="H6" s="10" t="str">
-        <x:v>Abarrotes</x:v>
+        <x:v>Harinas, mezclas y panificación</x:v>
       </x:c>
       <x:c r="I6" s="11" t="str"/>
       <x:c r="J6" s="10" t="str">
@@ -7130,7 +7156,7 @@
         <x:v>Hoy muestra y guarda UN; factor configurado 1:1.</x:v>
       </x:c>
       <x:c r="H7" s="10" t="str">
-        <x:v>Té</x:v>
+        <x:v>Té e infusiones</x:v>
       </x:c>
       <x:c r="I7" s="11" t="str"/>
       <x:c r="J7" s="10" t="str">
@@ -7166,7 +7192,7 @@
         <x:v>Hoy muestra y guarda UN; factor configurado 1:1.</x:v>
       </x:c>
       <x:c r="H8" s="10" t="str">
-        <x:v>Té</x:v>
+        <x:v>Té e infusiones</x:v>
       </x:c>
       <x:c r="I8" s="11" t="str"/>
       <x:c r="J8" s="10" t="str">
@@ -7202,7 +7228,7 @@
         <x:v>Hoy muestra y guarda UN; factor configurado 1:1.</x:v>
       </x:c>
       <x:c r="H9" s="10" t="str">
-        <x:v>Bebestibles</x:v>
+        <x:v>Rotulación y operación</x:v>
       </x:c>
       <x:c r="I9" s="11" t="str"/>
       <x:c r="J9" s="10" t="str">
@@ -7238,11 +7264,9 @@
         <x:v>Hoy muestra y guarda KG; factor configurado 1:1.</x:v>
       </x:c>
       <x:c r="H10" s="10" t="str">
-        <x:v>Bebestibles</x:v>
-      </x:c>
-      <x:c r="I10" s="11" t="str">
-        <x:v>Refrigerados y congelados</x:v>
-      </x:c>
+        <x:v>Helados, pulpas y congelados</x:v>
+      </x:c>
+      <x:c r="I10" s="11"/>
       <x:c r="J10" s="10" t="str">
         <x:v>No figura en el listado manual de Principal. ¿Bodega guarda esta pulpa y debe contarla? ¿Dónde se guarda?</x:v>
       </x:c>
@@ -7276,11 +7300,9 @@
         <x:v>Hoy muestra y guarda UN; factor configurado 1:1.</x:v>
       </x:c>
       <x:c r="H11" s="10" t="str">
-        <x:v>Carnes y Aves</x:v>
-      </x:c>
-      <x:c r="I11" s="11" t="str">
-        <x:v>Refrigerados y congelados</x:v>
-      </x:c>
+        <x:v>Carnes, aves y pescados</x:v>
+      </x:c>
+      <x:c r="I11" s="11"/>
       <x:c r="J11" s="10" t="str">
         <x:v>No figura en el listado manual de Principal. ¿Bodega guarda este producto y debe contarlo? ¿Dónde se guarda?</x:v>
       </x:c>
@@ -7314,11 +7336,9 @@
         <x:v>Hoy muestra y guarda KG; factor configurado 1:1.</x:v>
       </x:c>
       <x:c r="H12" s="10" t="str">
-        <x:v>Lácteos y Quesos</x:v>
-      </x:c>
-      <x:c r="I12" s="11" t="str">
-        <x:v>Refrigerados y congelados</x:v>
-      </x:c>
+        <x:v>Lácteos, cremas y grasas</x:v>
+      </x:c>
+      <x:c r="I12" s="11"/>
       <x:c r="J12" s="10" t="str">
         <x:v>No figura en el listado manual de Principal. ¿Bodega guarda este producto y debe contarlo? ¿Dónde se guarda?</x:v>
       </x:c>
@@ -7352,11 +7372,9 @@
         <x:v>Hoy muestra y guarda KG; factor configurado 1:1.</x:v>
       </x:c>
       <x:c r="H13" s="10" t="str">
-        <x:v>Lácteos y Quesos</x:v>
-      </x:c>
-      <x:c r="I13" s="11" t="str">
-        <x:v>Refrigerados y congelados</x:v>
-      </x:c>
+        <x:v>Lácteos, cremas y grasas</x:v>
+      </x:c>
+      <x:c r="I13" s="11"/>
       <x:c r="J13" s="10" t="str">
         <x:v>No figura en el listado manual de Principal. ¿Bodega guarda este producto y debe contarlo? ¿Dónde se guarda?</x:v>
       </x:c>
@@ -7669,7 +7687,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R57d0d85ebc7a47d6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8d311db07f944234"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>